<commit_message>
Lots of work on Figures
Fine-tuning figures as I finish first draft of manuscript.
</commit_message>
<xml_diff>
--- a/results-raw/Dsuite/Pcra_dsuite_results_combined.xlsx
+++ b/results-raw/Dsuite/Pcra_dsuite_results_combined.xlsx
@@ -1,26 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Shared/KKMDocuments/Documents/Github.Repos/Pcra/Pcra_phylogenetics/results-raw/Dsuite/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D49A44D-7982-CE43-9172-86EB5DA168CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09550544-BDC3-024E-BB92-0BF76A162188}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6560" yWindow="7820" windowWidth="28040" windowHeight="17440" xr2:uid="{FCB3DC1D-6121-EB49-A21A-B18172037AEC}"/>
+    <workbookView xWindow="33040" yWindow="500" windowWidth="28040" windowHeight="17440" activeTab="1" xr2:uid="{FCB3DC1D-6121-EB49-A21A-B18172037AEC}"/>
   </bookViews>
   <sheets>
     <sheet name="Pcra_dsuite_results_combined_tr" sheetId="1" r:id="rId1"/>
+    <sheet name="For manuscript" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="26">
   <si>
     <t>P1</t>
   </si>
@@ -92,12 +93,21 @@
   </si>
   <si>
     <t>Sample name</t>
+  </si>
+  <si>
+    <t>SFPW N. Atlantic</t>
+  </si>
+  <si>
+    <t>FKW N. Atlantic</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.000"/>
+  </numFmts>
   <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -575,9 +585,11 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1675,4 +1687,694 @@
   </sortState>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C399DF9C-47CD-884B-A09C-C7077ADB0F5F}">
+  <dimension ref="A1:J21"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="3" width="14.83203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2" s="3">
+        <v>6.08338E-2</v>
+      </c>
+      <c r="E2" s="2">
+        <v>10.4704</v>
+      </c>
+      <c r="F2" s="1">
+        <v>2.2999999999999999E-16</v>
+      </c>
+      <c r="G2" s="3">
+        <v>7.4876600000000001E-2</v>
+      </c>
+      <c r="H2">
+        <v>492187</v>
+      </c>
+      <c r="I2">
+        <v>498290</v>
+      </c>
+      <c r="J2">
+        <v>441140</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" s="3">
+        <v>0.10276299999999999</v>
+      </c>
+      <c r="E3" s="2">
+        <v>17.125</v>
+      </c>
+      <c r="F3" s="1">
+        <v>2.2999999999999999E-16</v>
+      </c>
+      <c r="G3" s="3">
+        <v>8.0960800000000003E-3</v>
+      </c>
+      <c r="H3" s="1">
+        <v>3863690</v>
+      </c>
+      <c r="I3">
+        <v>200197</v>
+      </c>
+      <c r="J3">
+        <v>162886</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D4" s="3">
+        <v>9.3257900000000005E-2</v>
+      </c>
+      <c r="E4" s="2">
+        <v>16.2761</v>
+      </c>
+      <c r="F4" s="1">
+        <v>2.2999999999999999E-16</v>
+      </c>
+      <c r="G4" s="3">
+        <v>7.5061900000000003E-3</v>
+      </c>
+      <c r="H4" s="1">
+        <v>3940270</v>
+      </c>
+      <c r="I4">
+        <v>195430</v>
+      </c>
+      <c r="J4">
+        <v>162089</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" s="3">
+        <v>9.4140799999999997E-2</v>
+      </c>
+      <c r="E5" s="2">
+        <v>15.597099999999999</v>
+      </c>
+      <c r="F5" s="1">
+        <v>2.2999999999999999E-16</v>
+      </c>
+      <c r="G5" s="3">
+        <v>7.4846599999999998E-3</v>
+      </c>
+      <c r="H5" s="1">
+        <v>3906830</v>
+      </c>
+      <c r="I5">
+        <v>196690</v>
+      </c>
+      <c r="J5">
+        <v>162843</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" s="3">
+        <v>4.4516500000000001E-2</v>
+      </c>
+      <c r="E6" s="2">
+        <v>8.0365699999999993</v>
+      </c>
+      <c r="F6" s="1">
+        <v>9.23849E-16</v>
+      </c>
+      <c r="G6" s="3">
+        <v>3.6859499999999999E-3</v>
+      </c>
+      <c r="H6" s="1">
+        <v>3821210</v>
+      </c>
+      <c r="I6">
+        <v>198778</v>
+      </c>
+      <c r="J6">
+        <v>181834</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D7" s="3">
+        <v>3.7398300000000002E-2</v>
+      </c>
+      <c r="E7" s="2">
+        <v>7.4960399999999998</v>
+      </c>
+      <c r="F7" s="1">
+        <v>6.5775299999999999E-14</v>
+      </c>
+      <c r="G7" s="3">
+        <v>3.1581999999999999E-3</v>
+      </c>
+      <c r="H7" s="1">
+        <v>3894800</v>
+      </c>
+      <c r="I7">
+        <v>194057</v>
+      </c>
+      <c r="J7">
+        <v>180065</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D8" s="3">
+        <v>3.8527400000000003E-2</v>
+      </c>
+      <c r="E8" s="2">
+        <v>7.3445999999999998</v>
+      </c>
+      <c r="F8" s="1">
+        <v>2.06381E-13</v>
+      </c>
+      <c r="G8" s="3">
+        <v>3.2146800000000001E-3</v>
+      </c>
+      <c r="H8" s="1">
+        <v>3862570</v>
+      </c>
+      <c r="I8">
+        <v>195403</v>
+      </c>
+      <c r="J8">
+        <v>180905</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>25</v>
+      </c>
+      <c r="B9" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" s="3">
+        <v>5.5972099999999997E-2</v>
+      </c>
+      <c r="E9" s="2">
+        <v>11.481999999999999</v>
+      </c>
+      <c r="F9" s="1">
+        <v>2.2999999999999999E-16</v>
+      </c>
+      <c r="G9" s="3">
+        <v>4.4552100000000002E-3</v>
+      </c>
+      <c r="H9" s="1">
+        <v>3867640</v>
+      </c>
+      <c r="I9">
+        <v>193203</v>
+      </c>
+      <c r="J9">
+        <v>172722</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D10" s="3">
+        <v>5.3881499999999999E-2</v>
+      </c>
+      <c r="E10" s="2">
+        <v>11.608599999999999</v>
+      </c>
+      <c r="F10" s="1">
+        <v>2.2999999999999999E-16</v>
+      </c>
+      <c r="G10" s="3">
+        <v>4.3847900000000004E-3</v>
+      </c>
+      <c r="H10" s="1">
+        <v>3946890</v>
+      </c>
+      <c r="I10">
+        <v>190088</v>
+      </c>
+      <c r="J10">
+        <v>170651</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11" t="s">
+        <v>20</v>
+      </c>
+      <c r="C11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D11" s="3">
+        <v>5.3930100000000002E-2</v>
+      </c>
+      <c r="E11" s="2">
+        <v>12.007300000000001</v>
+      </c>
+      <c r="F11" s="1">
+        <v>2.2999999999999999E-16</v>
+      </c>
+      <c r="G11" s="3">
+        <v>4.3282800000000003E-3</v>
+      </c>
+      <c r="H11" s="1">
+        <v>3912720</v>
+      </c>
+      <c r="I11">
+        <v>190847</v>
+      </c>
+      <c r="J11">
+        <v>171316</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D12" s="3">
+        <v>0.14274400000000001</v>
+      </c>
+      <c r="E12" s="2">
+        <v>25.880700000000001</v>
+      </c>
+      <c r="F12" s="1">
+        <v>2.2999999999999999E-16</v>
+      </c>
+      <c r="G12" s="3">
+        <v>1.8088300000000002E-2</v>
+      </c>
+      <c r="H12" s="1">
+        <v>3373250</v>
+      </c>
+      <c r="I12">
+        <v>328638</v>
+      </c>
+      <c r="J12">
+        <v>246536</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>17</v>
+      </c>
+      <c r="B13" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13" t="s">
+        <v>21</v>
+      </c>
+      <c r="D13" s="3">
+        <v>0.136515</v>
+      </c>
+      <c r="E13" s="2">
+        <v>21.164400000000001</v>
+      </c>
+      <c r="F13" s="1">
+        <v>2.2999999999999999E-16</v>
+      </c>
+      <c r="G13" s="3">
+        <v>1.6589199999999998E-2</v>
+      </c>
+      <c r="H13" s="1">
+        <v>3390170</v>
+      </c>
+      <c r="I13">
+        <v>310333</v>
+      </c>
+      <c r="J13">
+        <v>235780</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>17</v>
+      </c>
+      <c r="B14" t="s">
+        <v>16</v>
+      </c>
+      <c r="C14" t="s">
+        <v>25</v>
+      </c>
+      <c r="D14" s="3">
+        <v>0.14063300000000001</v>
+      </c>
+      <c r="E14" s="2">
+        <v>23.078900000000001</v>
+      </c>
+      <c r="F14" s="1">
+        <v>2.2999999999999999E-16</v>
+      </c>
+      <c r="G14" s="3">
+        <v>1.7416500000000001E-2</v>
+      </c>
+      <c r="H14" s="1">
+        <v>3382370</v>
+      </c>
+      <c r="I14">
+        <v>318693</v>
+      </c>
+      <c r="J14">
+        <v>240108</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>17</v>
+      </c>
+      <c r="B15" t="s">
+        <v>24</v>
+      </c>
+      <c r="C15" t="s">
+        <v>20</v>
+      </c>
+      <c r="D15" s="3">
+        <v>6.3098199999999993E-2</v>
+      </c>
+      <c r="E15" s="2">
+        <v>13.411099999999999</v>
+      </c>
+      <c r="F15" s="1">
+        <v>2.2999999999999999E-16</v>
+      </c>
+      <c r="G15" s="3">
+        <v>7.6693500000000001E-3</v>
+      </c>
+      <c r="H15" s="1">
+        <v>3596410</v>
+      </c>
+      <c r="I15">
+        <v>293709</v>
+      </c>
+      <c r="J15">
+        <v>258844</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>17</v>
+      </c>
+      <c r="B16" t="s">
+        <v>24</v>
+      </c>
+      <c r="C16" t="s">
+        <v>21</v>
+      </c>
+      <c r="D16" s="3">
+        <v>6.2651299999999993E-2</v>
+      </c>
+      <c r="E16" s="2">
+        <v>17.1586</v>
+      </c>
+      <c r="F16" s="1">
+        <v>2.2999999999999999E-16</v>
+      </c>
+      <c r="G16" s="3">
+        <v>7.3072900000000001E-3</v>
+      </c>
+      <c r="H16" s="1">
+        <v>3610490</v>
+      </c>
+      <c r="I16">
+        <v>278876</v>
+      </c>
+      <c r="J16">
+        <v>245992</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>17</v>
+      </c>
+      <c r="B17" t="s">
+        <v>24</v>
+      </c>
+      <c r="C17" t="s">
+        <v>25</v>
+      </c>
+      <c r="D17" s="3">
+        <v>6.2680700000000006E-2</v>
+      </c>
+      <c r="E17" s="2">
+        <v>14.7506</v>
+      </c>
+      <c r="F17" s="1">
+        <v>2.2999999999999999E-16</v>
+      </c>
+      <c r="G17" s="3">
+        <v>7.4478399999999998E-3</v>
+      </c>
+      <c r="H17" s="1">
+        <v>3603930</v>
+      </c>
+      <c r="I17">
+        <v>285261</v>
+      </c>
+      <c r="J17">
+        <v>251610</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>24</v>
+      </c>
+      <c r="C18" t="s">
+        <v>16</v>
+      </c>
+      <c r="D18" s="3">
+        <v>4.0254899999999996E-3</v>
+      </c>
+      <c r="E18" s="2">
+        <v>0.54494500000000001</v>
+      </c>
+      <c r="F18" s="3">
+        <v>0.58579099999999995</v>
+      </c>
+      <c r="G18" s="3">
+        <v>3.3197700000000001E-3</v>
+      </c>
+      <c r="H18">
+        <v>837009</v>
+      </c>
+      <c r="I18">
+        <v>633013</v>
+      </c>
+      <c r="J18">
+        <v>627937</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>24</v>
+      </c>
+      <c r="B19" t="s">
+        <v>16</v>
+      </c>
+      <c r="C19" t="s">
+        <v>20</v>
+      </c>
+      <c r="D19" s="3">
+        <v>8.6154900000000006E-2</v>
+      </c>
+      <c r="E19" s="2">
+        <v>14.184699999999999</v>
+      </c>
+      <c r="F19" s="1">
+        <v>2.2999999999999999E-16</v>
+      </c>
+      <c r="G19" s="3">
+        <v>1.0463E-2</v>
+      </c>
+      <c r="H19" s="1">
+        <v>3346180</v>
+      </c>
+      <c r="I19">
+        <v>297007</v>
+      </c>
+      <c r="J19">
+        <v>249889</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>24</v>
+      </c>
+      <c r="B20" t="s">
+        <v>16</v>
+      </c>
+      <c r="C20" t="s">
+        <v>21</v>
+      </c>
+      <c r="D20" s="3">
+        <v>7.9997600000000002E-2</v>
+      </c>
+      <c r="E20" s="2">
+        <v>12.4915</v>
+      </c>
+      <c r="F20" s="1">
+        <v>2.2999999999999999E-16</v>
+      </c>
+      <c r="G20" s="3">
+        <v>9.3261799999999999E-3</v>
+      </c>
+      <c r="H20" s="1">
+        <v>3363490</v>
+      </c>
+      <c r="I20">
+        <v>280803</v>
+      </c>
+      <c r="J20">
+        <v>239204</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>24</v>
+      </c>
+      <c r="B21" t="s">
+        <v>16</v>
+      </c>
+      <c r="C21" t="s">
+        <v>25</v>
+      </c>
+      <c r="D21" s="3">
+        <v>8.4375099999999995E-2</v>
+      </c>
+      <c r="E21" s="2">
+        <v>13.4871</v>
+      </c>
+      <c r="F21" s="1">
+        <v>2.2999999999999999E-16</v>
+      </c>
+      <c r="G21" s="3">
+        <v>1.00258E-2</v>
+      </c>
+      <c r="H21" s="1">
+        <v>3355370</v>
+      </c>
+      <c r="I21">
+        <v>288474</v>
+      </c>
+      <c r="J21">
+        <v>243582</v>
+      </c>
+    </row>
+  </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J21">
+    <sortCondition ref="A2:A21"/>
+    <sortCondition ref="B2:B21"/>
+    <sortCondition ref="C2:C21"/>
+  </sortState>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>